<commit_message>
Add GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/FOMS生产主流程/其他/wave_numbers.xlsx
+++ b/FOMS生产主流程/其他/wave_numbers.xlsx
@@ -27,21 +27,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
     <t>wave_number</t>
   </si>
   <si>
-    <t>W003934091</t>
+    <t>W003948135</t>
   </si>
   <si>
-    <t>W003934090</t>
+    <t>W003948134</t>
   </si>
   <si>
-    <t>W003934089</t>
+    <t>W003948133</t>
   </si>
   <si>
-    <t>W003934088</t>
+    <t>W003948132</t>
   </si>
 </sst>
 </file>
@@ -1201,8 +1201,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14" outlineLevelRow="4"/>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14" outlineLevelRow="7"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
@@ -1221,11 +1221,26 @@
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>